<commit_message>
Upload the Excel table with graph
</commit_message>
<xml_diff>
--- a/Lab4/Lab4_ADC.xlsx
+++ b/Lab4/Lab4_ADC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/zmen433_uoa_auckland_ac_nz/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1253570-B1A1-4297-9E13-CAA2B0FC59BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="8_{C1253570-B1A1-4297-9E13-CAA2B0FC59BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2ABF311-BDB3-4802-856B-0EBA609DE51E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{70CC4A89-B884-421D-A23D-160A0FED6802}"/>
   </bookViews>
@@ -39,7 +39,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t>ADC0_mV</t>
+  </si>
+  <si>
+    <t>ADC1_mV</t>
+  </si>
+  <si>
+    <t>Sample</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -91,6 +101,1190 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$A$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ADC0_mV</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$41</c:f>
+              <c:numCache>
+                <c:formatCode>@</c:formatCode>
+                <c:ptCount val="40"/>
+                <c:pt idx="0">
+                  <c:v>997</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4354</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>513</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4389</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>943</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3553</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2086</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2218</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3426</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1041</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4340</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>513</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4408</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>904</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3582</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2043</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2306</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>3372</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1085</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4301</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>518</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>4423</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>869</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3646</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1930</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2399</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>3240</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1182</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>4247</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>527</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>4467</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>772</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>3758</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>1823</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>2536</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>3128</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>1265</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>4183</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>557</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>4481</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5A13-4A47-97A5-4DDF9A04EBA3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ADC1_mV</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$41</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="40"/>
+                <c:pt idx="0">
+                  <c:v>3377</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1847</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2854</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2492</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2189</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3113</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1652</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3479</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1510</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3382</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1827</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2873</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2463</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2199</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3088</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1681</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3475</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>1510</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3406</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1793</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2913</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>2424</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2243</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3069</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1705</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>3450</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>1505</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>3431</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>1749</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>2996</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>2321</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>2316</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>3010</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>1739</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>3431</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>1505</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>3450</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>1705</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>3044</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>2282</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5A13-4A47-97A5-4DDF9A04EBA3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1166934112"/>
+        <c:axId val="1009808752"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1166934112"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1009808752"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1009808752"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="@" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1166934112"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>461962</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>80962</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>233362</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>109537</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F86246B9-D06C-4B85-E318-A62DBE7577F2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -410,334 +1604,474 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CD53C74-478C-45F7-BAA0-A6D9E4DB0127}">
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="16.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.25" customWidth="1"/>
+    <col min="3" max="3" width="16.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1">
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1">
         <v>997</v>
       </c>
-      <c r="B1">
+      <c r="B2">
         <v>3377</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1">
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1">
         <v>4354</v>
       </c>
-      <c r="B2">
+      <c r="B3">
         <v>1847</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="1">
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="1">
         <v>513</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>2854</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="1">
+      <c r="C4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="1">
         <v>4389</v>
       </c>
-      <c r="B4">
+      <c r="B5">
         <v>2492</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="1">
+      <c r="C5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="1">
         <v>943</v>
       </c>
-      <c r="B5">
+      <c r="B6">
         <v>2189</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="1">
+      <c r="C6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="1">
         <v>3553</v>
       </c>
-      <c r="B6">
+      <c r="B7">
         <v>3113</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="1">
+      <c r="C7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="1">
         <v>2086</v>
       </c>
-      <c r="B7">
+      <c r="B8">
         <v>1652</v>
       </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="1">
+      <c r="C8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="1">
         <v>2218</v>
       </c>
-      <c r="B8">
+      <c r="B9">
         <v>3479</v>
       </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="1">
+      <c r="C9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="1">
         <v>3426</v>
       </c>
-      <c r="B9">
+      <c r="B10">
         <v>1510</v>
       </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="1">
+      <c r="C10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="1">
         <v>1041</v>
       </c>
-      <c r="B10">
+      <c r="B11">
         <v>3382</v>
       </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="1">
+      <c r="C11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="1">
         <v>4340</v>
       </c>
-      <c r="B11">
+      <c r="B12">
         <v>1827</v>
       </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="1">
+      <c r="C12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="1">
         <v>513</v>
       </c>
-      <c r="B12">
+      <c r="B13">
         <v>2873</v>
       </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="1">
+      <c r="C13">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="1">
         <v>4408</v>
       </c>
-      <c r="B13">
+      <c r="B14">
         <v>2463</v>
       </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="1">
+      <c r="C14">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="1">
         <v>904</v>
       </c>
-      <c r="B14">
+      <c r="B15">
         <v>2199</v>
       </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="1">
+      <c r="C15">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="1">
         <v>3582</v>
       </c>
-      <c r="B15">
+      <c r="B16">
         <v>3088</v>
       </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="1">
+      <c r="C16">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="1">
         <v>2043</v>
       </c>
-      <c r="B16">
+      <c r="B17">
         <v>1681</v>
       </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="1">
+      <c r="C17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="1">
         <v>2306</v>
       </c>
-      <c r="B17">
+      <c r="B18">
         <v>3475</v>
       </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="1">
+      <c r="C18">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="1">
         <v>3372</v>
       </c>
-      <c r="B18">
+      <c r="B19">
         <v>1510</v>
       </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="1">
+      <c r="C19">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="1">
         <v>1085</v>
       </c>
-      <c r="B19">
+      <c r="B20">
         <v>3406</v>
       </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="1">
+      <c r="C20">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="1">
         <v>4301</v>
       </c>
-      <c r="B20">
+      <c r="B21">
         <v>1793</v>
       </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="1">
+      <c r="C21">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="1">
         <v>518</v>
       </c>
-      <c r="B21">
+      <c r="B22">
         <v>2913</v>
       </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="1">
+      <c r="C22">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="1">
         <v>4423</v>
       </c>
-      <c r="B22">
+      <c r="B23">
         <v>2424</v>
       </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="1">
+      <c r="C23">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="1">
         <v>869</v>
       </c>
-      <c r="B23">
+      <c r="B24">
         <v>2243</v>
       </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="1">
+      <c r="C24">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="1">
         <v>3646</v>
       </c>
-      <c r="B24">
+      <c r="B25">
         <v>3069</v>
       </c>
-    </row>
-    <row r="25" spans="1:2">
-      <c r="A25" s="1">
+      <c r="C25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="1">
         <v>1930</v>
       </c>
-      <c r="B25">
+      <c r="B26">
         <v>1705</v>
       </c>
-    </row>
-    <row r="26" spans="1:2">
-      <c r="A26" s="1">
+      <c r="C26">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="1">
         <v>2399</v>
       </c>
-      <c r="B26">
+      <c r="B27">
         <v>3450</v>
       </c>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="A27" s="1">
+      <c r="C27">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" s="1">
         <v>3240</v>
       </c>
-      <c r="B27">
+      <c r="B28">
         <v>1505</v>
       </c>
-    </row>
-    <row r="28" spans="1:2">
-      <c r="A28" s="1">
+      <c r="C28">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" s="1">
         <v>1182</v>
       </c>
-      <c r="B28">
+      <c r="B29">
         <v>3431</v>
       </c>
-    </row>
-    <row r="29" spans="1:2">
-      <c r="A29" s="1">
+      <c r="C29">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="1">
         <v>4247</v>
       </c>
-      <c r="B29">
+      <c r="B30">
         <v>1749</v>
       </c>
-    </row>
-    <row r="30" spans="1:2">
-      <c r="A30" s="1">
+      <c r="C30">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" s="1">
         <v>527</v>
       </c>
-      <c r="B30">
+      <c r="B31">
         <v>2996</v>
       </c>
-    </row>
-    <row r="31" spans="1:2">
-      <c r="A31" s="1">
+      <c r="C31">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" s="1">
         <v>4467</v>
       </c>
-      <c r="B31">
+      <c r="B32">
         <v>2321</v>
       </c>
-    </row>
-    <row r="32" spans="1:2">
-      <c r="A32" s="1">
+      <c r="C32">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="1">
         <v>772</v>
       </c>
-      <c r="B32">
+      <c r="B33">
         <v>2316</v>
       </c>
-    </row>
-    <row r="33" spans="1:2">
-      <c r="A33" s="1">
+      <c r="C33">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="1">
         <v>3758</v>
       </c>
-      <c r="B33">
+      <c r="B34">
         <v>3010</v>
       </c>
-    </row>
-    <row r="34" spans="1:2">
-      <c r="A34" s="1">
+      <c r="C34">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="1">
         <v>1823</v>
       </c>
-      <c r="B34">
+      <c r="B35">
         <v>1739</v>
       </c>
-    </row>
-    <row r="35" spans="1:2">
-      <c r="A35" s="1">
+      <c r="C35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="1">
         <v>2536</v>
       </c>
-      <c r="B35">
+      <c r="B36">
         <v>3431</v>
       </c>
-    </row>
-    <row r="36" spans="1:2">
-      <c r="A36" s="1">
+      <c r="C36">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="1">
         <v>3128</v>
       </c>
-      <c r="B36">
+      <c r="B37">
         <v>1505</v>
       </c>
-    </row>
-    <row r="37" spans="1:2">
-      <c r="A37" s="1">
+      <c r="C37">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="1">
         <v>1265</v>
       </c>
-      <c r="B37">
+      <c r="B38">
         <v>3450</v>
       </c>
-    </row>
-    <row r="38" spans="1:2">
-      <c r="A38" s="1">
+      <c r="C38">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="1">
         <v>4183</v>
       </c>
-      <c r="B38">
+      <c r="B39">
         <v>1705</v>
       </c>
-    </row>
-    <row r="39" spans="1:2">
-      <c r="A39" s="1">
+      <c r="C39">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="1">
         <v>557</v>
       </c>
-      <c r="B39">
+      <c r="B40">
         <v>3044</v>
       </c>
-    </row>
-    <row r="40" spans="1:2">
-      <c r="A40" s="1">
+      <c r="C40">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="1">
         <v>4481</v>
       </c>
-      <c r="B40">
+      <c r="B41">
         <v>2282</v>
+      </c>
+      <c r="C41">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" enabled="0" method="" siteId="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>